<commit_message>
Requirements Datei geschlossen. Temp datei weg
</commit_message>
<xml_diff>
--- a/04_Aufgabe-Requirements/A/Requirements_MarvinBock.xlsx
+++ b/04_Aufgabe-Requirements/A/Requirements_MarvinBock.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Studium\Semester 4\Softwaretechnik\REPO\Softwaretechnik_MBock\04_Aufgabe-Requirements\A\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F68C49F1-7C7A-4437-8EE5-68DA2E81A624}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35393AB7-8966-4A55-839C-BCC9A8D2C9AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6255" yWindow="4665" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-25275" yWindow="4245" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -254,14 +254,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="3">
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -291,7 +300,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E0E7A0C0-7947-4BD6-B1F3-E4013431E52B}" name="Tabelle2" displayName="Tabelle2" ref="A1:K9" totalsRowShown="0" headerRowDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E0E7A0C0-7947-4BD6-B1F3-E4013431E52B}" name="Tabelle2" displayName="Tabelle2" ref="A1:K9" totalsRowShown="0" headerRowDxfId="2">
   <autoFilter ref="A1:K9" xr:uid="{E0E7A0C0-7947-4BD6-B1F3-E4013431E52B}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{9C6E35E3-B30B-494F-AABA-2758CF4518DB}" name="ID"/>
@@ -300,8 +309,8 @@
     <tableColumn id="4" xr3:uid="{CA446B89-ED80-42DB-A140-226524F20EFA}" name="Priorität"/>
     <tableColumn id="5" xr3:uid="{EDCD8751-58C1-44CE-8984-74F7B85403CF}" name="Status"/>
     <tableColumn id="6" xr3:uid="{8C674DCD-DD80-4ABA-B5EA-FCCC3FA91DF6}" name="Quelle"/>
-    <tableColumn id="7" xr3:uid="{91BC3A32-61DB-4363-8698-5FAD8CAA150B}" name="Beschreibung"/>
-    <tableColumn id="8" xr3:uid="{96E69B78-1AFD-46D8-8D1B-5E295BBBD79E}" name="Akzeptanzkriterium"/>
+    <tableColumn id="7" xr3:uid="{91BC3A32-61DB-4363-8698-5FAD8CAA150B}" name="Beschreibung" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{96E69B78-1AFD-46D8-8D1B-5E295BBBD79E}" name="Akzeptanzkriterium" dataDxfId="0"/>
     <tableColumn id="9" xr3:uid="{47260C11-D211-4257-B0CA-C8B47FB78387}" name="Risiko"/>
     <tableColumn id="10" xr3:uid="{D493DBC1-1C81-43A1-A83E-3A28CC441921}" name="Verantwortlich"/>
     <tableColumn id="11" xr3:uid="{CC93536C-5C95-41D5-9E05-DF80D7F0EA9B}" name="Version"/>
@@ -573,16 +582,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="32.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.42578125" customWidth="1"/>
     <col min="5" max="5" width="8.5703125" customWidth="1"/>
     <col min="6" max="6" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="80.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="60.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="41" customWidth="1"/>
+    <col min="8" max="8" width="37.140625" customWidth="1"/>
     <col min="9" max="9" width="8.5703125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="23.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="10" customWidth="1"/>
@@ -623,7 +636,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -642,10 +655,10 @@
       <c r="F2" t="s">
         <v>16</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="2" t="s">
         <v>18</v>
       </c>
       <c r="I2" t="s">
@@ -658,7 +671,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>22</v>
       </c>
@@ -677,10 +690,10 @@
       <c r="F3" t="s">
         <v>16</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="2" t="s">
         <v>31</v>
       </c>
       <c r="I3" t="s">
@@ -693,7 +706,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>23</v>
       </c>
@@ -712,10 +725,10 @@
       <c r="F4" t="s">
         <v>16</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H4" s="2" t="s">
         <v>36</v>
       </c>
       <c r="I4" t="s">
@@ -728,7 +741,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>24</v>
       </c>
@@ -747,10 +760,10 @@
       <c r="F5" t="s">
         <v>16</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H5" s="2" t="s">
         <v>41</v>
       </c>
       <c r="I5" t="s">
@@ -763,7 +776,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -782,10 +795,10 @@
       <c r="F6" t="s">
         <v>45</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="H6" t="s">
+      <c r="H6" s="2" t="s">
         <v>47</v>
       </c>
       <c r="I6" t="s">
@@ -798,7 +811,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>26</v>
       </c>
@@ -817,10 +830,10 @@
       <c r="F7" t="s">
         <v>16</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="H7" t="s">
+      <c r="H7" s="2" t="s">
         <v>50</v>
       </c>
       <c r="I7" t="s">
@@ -833,7 +846,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>27</v>
       </c>
@@ -852,10 +865,10 @@
       <c r="F8" t="s">
         <v>57</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G8" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H8" t="s">
+      <c r="H8" s="2" t="s">
         <v>55</v>
       </c>
       <c r="I8" t="s">
@@ -868,7 +881,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>28</v>
       </c>
@@ -887,10 +900,10 @@
       <c r="F9" t="s">
         <v>57</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="H9" t="s">
+      <c r="H9" s="2" t="s">
         <v>59</v>
       </c>
       <c r="I9" t="s">
@@ -905,9 +918,10 @@
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="8" scale="91" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>